<commit_message>
Fix delete rows in formula widget; add PDR Lao demo instance
- formula_widget: extract collapse logic into review_df reactive shared
  by renderDT and deleteRows handler; when collapsed, delete by
  dataElement.id so all underlying category rows are removed correctly
- login_widget: add PDR Lao HMIS (demos.dhis2.org/hmis_data) as first
  demo option with demo_en / District1# credentials

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/shiny/Instances.xlsx
+++ b/inst/shiny/Instances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdc-my.sharepoint.com/personal/bzp3_cdc_gov/Documents/_Malaria/Projects/MagicGlasses2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnpainter/Library/Mobile Documents/com~apple~CloudDocs/Projects/MG2/inst/shiny/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{FAA29904-BAA7-F844-9D08-9E9F00116AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{433C3A1F-D414-4D5E-94A7-23DE0BE2FC06}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB2A801-B018-BF4E-9726-8C73CD3F989F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3345" yWindow="2505" windowWidth="21600" windowHeight="11385" xr2:uid="{8BA4FBCD-55B1-E647-B41A-02F2E5FD225B}"/>
+    <workbookView xWindow="3340" yWindow="2500" windowWidth="21600" windowHeight="11380" xr2:uid="{8BA4FBCD-55B1-E647-B41A-02F2E5FD225B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -54,19 +54,19 @@
     <t>DHIS2 Demo 2.40</t>
   </si>
   <si>
-    <t>https://play.dhis2.org/2.40/</t>
-  </si>
-  <si>
-    <t>DHIS2 Demo 2.39</t>
-  </si>
-  <si>
-    <t>https://play.dhis2.org/2.39/</t>
-  </si>
-  <si>
-    <t>DHIS2 Demo 2.38</t>
-  </si>
-  <si>
-    <t>https://play.dhis2.org/2.38/</t>
+    <t>https://play.im.dhis2.org/stable-2-42-4/dhis-web-login/</t>
+  </si>
+  <si>
+    <t>DHIS2 Demo 2.42</t>
+  </si>
+  <si>
+    <t>DHIS2 Demo 2.41</t>
+  </si>
+  <si>
+    <t>https://play.im.dhis2.org/stable-2-41-8/</t>
+  </si>
+  <si>
+    <t>https://play.im.dhis2.org/stable-2-40-11/</t>
   </si>
 </sst>
 </file>
@@ -139,9 +139,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -179,7 +179,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -285,7 +285,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -427,7 +427,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -436,13 +436,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D35E3C44-5FD4-CF47-9179-77B24E15A800}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="60.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -456,9 +456,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>7</v>
@@ -470,12 +470,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
@@ -484,9 +484,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>11</v>
@@ -502,10 +502,8 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{040B7DB1-B7CB-4A76-A93B-F5D9145BF95C}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{0F12C359-025B-45E9-9705-68F4D3BDA36D}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{3B1EE631-E85C-4C9F-B3CD-45EC4D474670}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>